<commit_message>
Update SKU Parasum stock data
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SKU PARASUM.xlsx
+++ b/SKU PARASUM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcajaravilla\Desktop\Proyectos Antigravity\parasum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEB2CF8-C6F5-4BF7-B7DE-0DB227F794B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02DE2EC-8EB2-4EBF-AE45-1B57637336F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PL3" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PL2'!$D$1:$D$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PL3'!$D$1:$D$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PL3'!$A$1:$D$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="296">
   <si>
     <t>Codigo</t>
   </si>
@@ -112,12 +112,6 @@
     <t>91AS12HR4SVRKG03PX4E</t>
   </si>
   <si>
-    <t>AIRE ACOND. HISENSE SPLIT 8000W FRIO CALOR CL. A (U.E.)</t>
-  </si>
-  <si>
-    <t>Aire 8000W</t>
-  </si>
-  <si>
     <t>91AS12HR4SVRKG03PX4I</t>
   </si>
   <si>
@@ -127,12 +121,6 @@
     <t>Otros</t>
   </si>
   <si>
-    <t>PAVA ELECTRICA CON CORTE SANSEI</t>
-  </si>
-  <si>
-    <t>Pava</t>
-  </si>
-  <si>
     <t>SMART TV 40" PHILCO - VIDAA</t>
   </si>
   <si>
@@ -163,63 +151,9 @@
     <t>Freezer 65L</t>
   </si>
   <si>
-    <t>Generador Electrico 2500W</t>
-  </si>
-  <si>
-    <t>Generador 2500W</t>
-  </si>
-  <si>
-    <t>Horno grill 70 litros</t>
-  </si>
-  <si>
-    <t>Horno 70L</t>
-  </si>
-  <si>
     <t>91ASGEN2</t>
   </si>
   <si>
-    <t>HORNO DE PAN ATMA NEGRO</t>
-  </si>
-  <si>
-    <t>Horno</t>
-  </si>
-  <si>
-    <t>LAVAVAJILLA HISENSE INOX 14 CUBIERTOS</t>
-  </si>
-  <si>
-    <t>Lavavajillas 14</t>
-  </si>
-  <si>
-    <t>Juguera negra PHILCO</t>
-  </si>
-  <si>
-    <t>Juguera</t>
-  </si>
-  <si>
-    <t>LAVAVAJILLAS 5 CUBIERTOS - ATMA - NEGRO</t>
-  </si>
-  <si>
-    <t>Lavavajillas 5</t>
-  </si>
-  <si>
-    <t>microondas Atma Digital C/ grill Black 23 Membrana</t>
-  </si>
-  <si>
-    <t>Microondas</t>
-  </si>
-  <si>
-    <t>BICICLETA MTB ACERO 29 FIERCE F210 21VEL GRIS TALLE 18</t>
-  </si>
-  <si>
-    <t>Bicicleta</t>
-  </si>
-  <si>
-    <t>MOPA CENTRIFUGA CON RUEDAS Y PEDAL PROLINE</t>
-  </si>
-  <si>
-    <t>Mopa</t>
-  </si>
-  <si>
     <t>CALEFÓN PHILCO 14/L MIN - BLANCO - TIRO FORZADO - TECNOLOGÍA PILOTLESS</t>
   </si>
   <si>
@@ -232,24 +166,6 @@
     <t>Cava 12</t>
   </si>
   <si>
-    <t>LAVARROPA CARGA FRONTAL INVERTER 11KG 1400 RPM PHILCO PHLF1114BI</t>
-  </si>
-  <si>
-    <t>Lavarropas 11kg</t>
-  </si>
-  <si>
-    <t>TORRE DE LAVADO CARGA FRONTAL LAVARROPAS + LAVASECARROPA PHILCO DARK GRAY</t>
-  </si>
-  <si>
-    <t>Lavasecarropas</t>
-  </si>
-  <si>
-    <t>HELADERA SIDE BY SIDE 428L NETA NEGRA PHILCO - PHSB450N</t>
-  </si>
-  <si>
-    <t>Heladera 428L</t>
-  </si>
-  <si>
     <t>HELADERA SBS CROSSDOOR 385L NETOS CON DISPENSER + INVERTER INOX PHILCO - PHSB470XD2</t>
   </si>
   <si>
@@ -274,18 +190,6 @@
     <t>Heladera 179L</t>
   </si>
   <si>
-    <t>INODORO SMART SANSEI MIZU BLANCO</t>
-  </si>
-  <si>
-    <t>Inodoro</t>
-  </si>
-  <si>
-    <t>VENTILADOR DE TECHO 56"</t>
-  </si>
-  <si>
-    <t>Ventilador 56"</t>
-  </si>
-  <si>
     <t>Tostadora Blanca ATMA</t>
   </si>
   <si>
@@ -295,129 +199,51 @@
     <t>91PLD40HS24</t>
   </si>
   <si>
-    <t>Termotanque eléctrico SIAM 35lts TSI-TS035BM BLANCO</t>
-  </si>
-  <si>
-    <t>Termotanque 35L</t>
-  </si>
-  <si>
-    <t>Termotanque eléctrico SIAM 65lts TSI-TS065BM BLANCO</t>
-  </si>
-  <si>
-    <t>Termotanque 65L</t>
-  </si>
-  <si>
     <t>LAVARROPAS INVERTER LG BLANCO WM10WVC4S6 CON AI DD¿ Y THINQ 10KG 1400 RPM</t>
   </si>
   <si>
     <t>Lavarropas 10kg</t>
   </si>
   <si>
-    <t>ZRAY KAYAK 1 PERSONA</t>
-  </si>
-  <si>
-    <t>Kayak</t>
-  </si>
-  <si>
-    <t>INDOOR UNIT MULTIV CASSETTE 4 WAY 36 KBTU</t>
-  </si>
-  <si>
-    <t>Aire Industrial</t>
-  </si>
-  <si>
     <t>FREEZER HORIZONTAL HISENSE 297L</t>
   </si>
   <si>
     <t>Freezer 297L</t>
   </si>
   <si>
-    <t>CAJA ORGANIZADORA ATMA HOME</t>
-  </si>
-  <si>
-    <t>Organizador</t>
-  </si>
-  <si>
     <t>Freezer Vertical SIAM 181 litros FSI-CV181B</t>
   </si>
   <si>
     <t>Freezer 181L</t>
   </si>
   <si>
-    <t>FREEZER VERTICAL HISENSE BLANCO 82L</t>
-  </si>
-  <si>
-    <t>Freezer 82L</t>
-  </si>
-  <si>
-    <t>GUANTE DE BOXEO 10 OZ ROJO</t>
-  </si>
-  <si>
-    <t>Guante 10oz</t>
-  </si>
-  <si>
     <t>91SAS25HA4CNE</t>
   </si>
   <si>
-    <t>VENDA DE BOXEO 4 METROS NEGRO</t>
-  </si>
-  <si>
-    <t>Venda de Boxeo</t>
-  </si>
-  <si>
     <t>HORNO GRILL AIR FRYER ATMA 17 LITROS</t>
   </si>
   <si>
     <t>Freidora 17L</t>
   </si>
   <si>
-    <t>HELADERA BAJO MESADA 83L PLATA SIAM - HSI-BM093P2</t>
-  </si>
-  <si>
-    <t>Heladera 83L</t>
-  </si>
-  <si>
     <t>HELADERA BAJO MESADA 50L CORAL - SIAM RETRO HSI-BM50BR2</t>
   </si>
   <si>
     <t>Heladera 50L</t>
   </si>
   <si>
-    <t>Exhibidora vertical SIAM 65 litros HSI-EV065B2</t>
-  </si>
-  <si>
-    <t>Exhibidora 65L</t>
-  </si>
-  <si>
     <t>LAVAVAJILLAS 15 CUBIERTOS INOX</t>
   </si>
   <si>
     <t>Lavavajillas 15</t>
   </si>
   <si>
-    <t>Microondas Philco Digital blanco 23 lts</t>
-  </si>
-  <si>
-    <t>Microondas 23L</t>
-  </si>
-  <si>
-    <t>Soporte Movil Marca Philco Serie G</t>
-  </si>
-  <si>
-    <t>Soporte movil</t>
-  </si>
-  <si>
     <t>Cava termoeléctrica de vinos 28 Botellas PHILCO PHCAV028N</t>
   </si>
   <si>
     <t>Cava 28</t>
   </si>
   <si>
-    <t>Cava eléctrica con compresor 52 Botellas PHILCO PHCAV052N</t>
-  </si>
-  <si>
-    <t>Cava 52</t>
-  </si>
-  <si>
     <t>FREEZER POZO BLANCO PHILCO - PHCH144B</t>
   </si>
   <si>
@@ -448,30 +274,12 @@
     <t>Heladera 339L</t>
   </si>
   <si>
-    <t>AIRE ACONDICIONADO PHILCO PORTATIL 2650 W F/C</t>
-  </si>
-  <si>
-    <t>Aire 2650W</t>
-  </si>
-  <si>
-    <t>AIRE ACONDICIONADO PHILCO PORTATIL 3500 W F/C</t>
-  </si>
-  <si>
-    <t>Aire 3500W</t>
-  </si>
-  <si>
     <t>HELADERA HISENSE TOP MOUNT NO FROST INVERTER INOX 320L</t>
   </si>
   <si>
     <t>Heladera 320L</t>
   </si>
   <si>
-    <t>Lavasecarropa Hisense Carga Frontal 10/6kg Inverter</t>
-  </si>
-  <si>
-    <t>Lavasecarropas 6kg</t>
-  </si>
-  <si>
     <t>92PHCA14B</t>
   </si>
   <si>
@@ -517,9 +325,6 @@
     <t>Aire 2750W</t>
   </si>
   <si>
-    <t>91AS30HR4SBBTG00E</t>
-  </si>
-  <si>
     <t>MICROONDAS LG INVERTIR 42 LITROS NEO CHEFF NEGRO ESPEJADO</t>
   </si>
   <si>
@@ -538,9 +343,6 @@
     <t>Heladera 198L</t>
   </si>
   <si>
-    <t>91PE1821BP</t>
-  </si>
-  <si>
     <t>Plancha Seca PHILCO</t>
   </si>
   <si>
@@ -691,21 +493,12 @@
     <t>Lavarropas 9.5kg</t>
   </si>
   <si>
-    <t>92HS642D90X</t>
-  </si>
-  <si>
     <t>LAVARROPAS HISENSE 6KG TITANIUM CARGA SUPERIOR</t>
   </si>
   <si>
     <t>Lavarropas 6kg</t>
   </si>
   <si>
-    <t>92MATDGB23UAP</t>
-  </si>
-  <si>
-    <t>92MPCHLVA01PI</t>
-  </si>
-  <si>
     <t>AIRE ACOND. WHIRLPOOL SPLIT INVERTER 3000 FRIO CALOR CL. A (U.I.)</t>
   </si>
   <si>
@@ -802,51 +595,21 @@
     <t>92PHSB470XD2</t>
   </si>
   <si>
-    <t>9434185K1</t>
-  </si>
-  <si>
-    <t>94ARNU36GTAB4-ANWBLAT</t>
-  </si>
-  <si>
     <t>94CF3N297NEW</t>
   </si>
   <si>
-    <t>94COAH17PI</t>
-  </si>
-  <si>
     <t>94FSI-CV181B</t>
   </si>
   <si>
-    <t>94FV1N81NAW</t>
-  </si>
-  <si>
-    <t>94GB-BX2010BOX10R</t>
-  </si>
-  <si>
-    <t>94GB-BX20184MB</t>
-  </si>
-  <si>
-    <t>94HSI-BM093P2</t>
-  </si>
-  <si>
     <t>94HSI-BM50BR2</t>
   </si>
   <si>
-    <t>94HSI-EV065B2</t>
-  </si>
-  <si>
     <t>94LSI-LJ15X</t>
   </si>
   <si>
-    <t>94MPHDW23UAP</t>
-  </si>
-  <si>
     <t>94PHCAV028N</t>
   </si>
   <si>
-    <t>94PHCAV052N</t>
-  </si>
-  <si>
     <t>94PHCH144B</t>
   </si>
   <si>
@@ -862,18 +625,9 @@
     <t>94PHNC382XT</t>
   </si>
   <si>
-    <t>94PHP26HC9AN</t>
-  </si>
-  <si>
-    <t>94PHP35HC7AN</t>
-  </si>
-  <si>
     <t>94RT3N320NMC</t>
   </si>
   <si>
-    <t>94WDQY1014T</t>
-  </si>
-  <si>
     <t>94RC-67WSG</t>
   </si>
   <si>
@@ -913,74 +667,278 @@
     <t>94FSI-CV065B</t>
   </si>
   <si>
-    <t>92GE-PH2500ALP</t>
-  </si>
-  <si>
-    <t>92HG7022P</t>
-  </si>
-  <si>
-    <t>92HPAT24BP</t>
-  </si>
-  <si>
-    <t>92JUPH21BP</t>
-  </si>
-  <si>
-    <t>92LLJ05N</t>
-  </si>
-  <si>
-    <t>92MMFIF210GRISP</t>
-  </si>
-  <si>
     <t>94PHCAV012N</t>
   </si>
   <si>
-    <t>92PHLF1114BI</t>
-  </si>
-  <si>
-    <t>92PHLFT157GT</t>
-  </si>
-  <si>
-    <t>92PHSB450N</t>
-  </si>
-  <si>
-    <t>92PHSD179BD2</t>
-  </si>
-  <si>
-    <t>94PHTE080B2</t>
-  </si>
-  <si>
     <t>92RL230WW4AU</t>
   </si>
   <si>
-    <t>92SAMZINSC1API</t>
-  </si>
-  <si>
-    <t>92TEB5634LP</t>
-  </si>
-  <si>
     <t>94TO20WP</t>
   </si>
   <si>
-    <t>92TSI-TS035BM</t>
-  </si>
-  <si>
-    <t>92TSI-TS065BM</t>
-  </si>
-  <si>
     <t>92WM10WVC4S6</t>
   </si>
   <si>
     <t>94HGFA1724UAP</t>
   </si>
   <si>
-    <t>94PG1443MPI</t>
+    <t>Código SKU</t>
+  </si>
+  <si>
+    <t>91AS12UR4SVRCA02BKNE</t>
+  </si>
+  <si>
+    <t>91AS18HR4SXSKG00PX4E</t>
+  </si>
+  <si>
+    <t>91NXIN35HA3BNE</t>
+  </si>
+  <si>
+    <t>94FR246ABP</t>
+  </si>
+  <si>
+    <t>94HRBF125B</t>
+  </si>
+  <si>
+    <t>92PHLF6510B2</t>
+  </si>
+  <si>
+    <t>94PHSD179BD2</t>
+  </si>
+  <si>
+    <t>92PHTE050B2</t>
+  </si>
+  <si>
+    <t>92PHTE080B2</t>
+  </si>
+  <si>
+    <t>94RT3N375NMC</t>
+  </si>
+  <si>
+    <t>94PHCAV08N2</t>
+  </si>
+  <si>
+    <t>94PHNC417XI</t>
+  </si>
+  <si>
+    <t>94RQ697HB</t>
+  </si>
+  <si>
+    <t>94RS-20DCS</t>
+  </si>
+  <si>
+    <t>94RT3N461NMC</t>
+  </si>
+  <si>
+    <t>Aire 3300W</t>
+  </si>
+  <si>
+    <t>Aire 5000W</t>
+  </si>
+  <si>
+    <t>Aire 3550W</t>
+  </si>
+  <si>
+    <t>Freidora de Aire</t>
+  </si>
+  <si>
+    <t>Heladera 123L</t>
+  </si>
+  <si>
+    <t>Lavarropas 6.5kg</t>
+  </si>
+  <si>
+    <t>Termotanque 50L</t>
+  </si>
+  <si>
+    <t>Heladera 375L</t>
+  </si>
+  <si>
+    <t>Cava 8</t>
+  </si>
+  <si>
+    <t>Heladera 374L</t>
+  </si>
+  <si>
+    <t>Heladera 640L</t>
+  </si>
+  <si>
+    <t>Freezer 169L</t>
+  </si>
+  <si>
+    <t>Heladera 461L</t>
+  </si>
+  <si>
+    <t>AIRE ACOND. HISENSE SPLIT INVERTER BLACK 3300W FRIO CALOR CL. A (U.E.)</t>
+  </si>
+  <si>
+    <t>AIRE ACOND. HISENSE SPLIT 5000W FRIO CALOR CL. A (U.E.)</t>
+  </si>
+  <si>
+    <t>AIRE ACOND. NOBLEX SPLIT INVERTER 3550W FRIO CALOR CL. A++ (U.E.)</t>
+  </si>
+  <si>
+    <t>FREIDORA DE AIRE CON VISOR NEGRA 6 LITROS</t>
+  </si>
+  <si>
+    <t>HELADERA BAJO MESADA 123 LITROS ( NEGRA)</t>
+  </si>
+  <si>
+    <t>Lavarropas carga frontal 6,5kg PHILCO - Blanco PHLF6510B2</t>
+  </si>
+  <si>
+    <t>termotanque eléctrico philco 2000w blanco 50 litros</t>
+  </si>
+  <si>
+    <t>HELADERA HISENSE TOP MOUNT NO FROST INOX INVERTER DISPENSER 375L</t>
+  </si>
+  <si>
+    <t>CAVA TERMOELECTRICA 8 BOTELLAS PHILCO - PHCAV08N2</t>
+  </si>
+  <si>
+    <t>HELADERA COMBI NO FROST INVERTER 374L INOX PHILCO - PHNC417XI</t>
+  </si>
+  <si>
+    <t>Heladera Cross Door Hisense Inverter + Smart Screen 640 litros</t>
+  </si>
+  <si>
+    <t>Freezer Vertical Hisense Plata 169 litros</t>
+  </si>
+  <si>
+    <t>HELADERA HISENSE TOP MOUNT NO FROST INVERTER INOX DISPENSER 461L</t>
+  </si>
+  <si>
+    <t>A05.000.000 / A19.000.000</t>
+  </si>
+  <si>
+    <t>A09.000.000 / B05.000.000 / B16.000.000 / B18.000.000 / REC.000.000</t>
+  </si>
+  <si>
+    <t>A03.000.000 / B06.000.000</t>
+  </si>
+  <si>
+    <t>A07.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000 / B16.000.000</t>
+  </si>
+  <si>
+    <t>A02.000.000 / B06.000.000</t>
+  </si>
+  <si>
+    <t>A16.000.000 / B06.000.000 / B17.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000 / B09.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000 / B07.000.000</t>
+  </si>
+  <si>
+    <t>B10.000.000</t>
+  </si>
+  <si>
+    <t>B07.000.000</t>
+  </si>
+  <si>
+    <t>B18.000.000</t>
+  </si>
+  <si>
+    <t>A17.000.000 / B06.000.000 / B18.000.000</t>
+  </si>
+  <si>
+    <t>A16.000.000 / B06.000.000 / B08.000.000</t>
+  </si>
+  <si>
+    <t>A07.000.000 / ANA.LIS.IS</t>
+  </si>
+  <si>
+    <t>A09.000.000 / PL4.000.000</t>
+  </si>
+  <si>
+    <t>A16.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000</t>
+  </si>
+  <si>
+    <t>A09.000.000 / B11.000.000 / CAL.000.000</t>
+  </si>
+  <si>
+    <t>A14.000.000 / B06.000.000 / SIN.000.000</t>
+  </si>
+  <si>
+    <t>B18.000.000 / REC.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000 / B10.000.000</t>
+  </si>
+  <si>
+    <t>B06.000.000 / B07.000.000 / SCR.OCA.SA</t>
+  </si>
+  <si>
+    <t>A08.000.000 / A11.000.000 / A12.000.000 / A16.000.000 / A17.000.000 / B09.000.000 / SIN.000.000</t>
+  </si>
+  <si>
+    <t>A07.000.000 / A08.000.000 / CAL.000.000</t>
+  </si>
+  <si>
+    <t>A16.000.000 / ANA.LIS.IS / B06.000.000 / B16.000.000</t>
+  </si>
+  <si>
+    <t>A17.000.000 / A18.000.000 / B12.000.000</t>
+  </si>
+  <si>
+    <t>A18.000.000 / B11.000.000</t>
+  </si>
+  <si>
+    <t>A08.000.000 / B07.000.000</t>
+  </si>
+  <si>
+    <t>A12.000.000</t>
+  </si>
+  <si>
+    <t>B04.000.000</t>
+  </si>
+  <si>
+    <t>A09.000.000</t>
+  </si>
+  <si>
+    <t>PL4.000.000</t>
+  </si>
+  <si>
+    <t>A08.000.000 / A10.000.000</t>
+  </si>
+  <si>
+    <t>B09.000.000 / SIN.000.000</t>
+  </si>
+  <si>
+    <t>A13.000.000</t>
+  </si>
+  <si>
+    <t>A08.000.000 / CAL.000.000</t>
+  </si>
+  <si>
+    <t>B01.000.000</t>
+  </si>
+  <si>
+    <t>SIN.000.000</t>
+  </si>
+  <si>
+    <t>A11.000.000</t>
+  </si>
+  <si>
+    <t>A17.000.000 / SCR.00.000</t>
+  </si>
+  <si>
+    <t>A12.000.000 / A13.000.000 / A17.000.000 / SIN.000.000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -995,8 +953,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1008,8 +978,13 @@
         <fgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5496"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1017,15 +992,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24204,1025 +24198,689 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.81640625" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="19.90625" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>277</v>
+      <c r="D1" s="2" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" t="str">
-        <f>VLOOKUP(A2,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A01.000.000</v>
+      <c r="A2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>253</v>
-      </c>
-      <c r="B3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D3" t="str">
-        <f>VLOOKUP(A3,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A04.000.000</v>
+      <c r="A3" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="str">
-        <f>VLOOKUP(A4,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A05.000.000</v>
+      <c r="A4" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>304</v>
-      </c>
-      <c r="B5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" t="str">
-        <f>VLOOKUP(A5,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A05.000.000</v>
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="str">
-        <f>VLOOKUP(A6,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A06.000.000</v>
+      <c r="D6" s="3" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>283</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="str">
-        <f>VLOOKUP(A7,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A07.000.000</v>
+      <c r="A7" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>266</v>
-      </c>
-      <c r="B8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" t="str">
-        <f>VLOOKUP(A8,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A08.000.000</v>
+      <c r="A8" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>274</v>
-      </c>
-      <c r="B9" t="s">
-        <v>138</v>
-      </c>
-      <c r="C9" t="s">
-        <v>139</v>
-      </c>
-      <c r="D9" t="str">
-        <f>VLOOKUP(A9,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A08.000.000</v>
+      <c r="A9" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>269</v>
-      </c>
-      <c r="B10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" t="s">
-        <v>129</v>
-      </c>
-      <c r="D10" t="str">
-        <f>VLOOKUP(A10,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>A09.000.000</v>
+      <c r="A10" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>264</v>
-      </c>
-      <c r="B11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C11" t="s">
-        <v>117</v>
-      </c>
-      <c r="D11" t="str">
-        <f>VLOOKUP(A11,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B01.000.000</v>
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>300</v>
-      </c>
-      <c r="B12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" t="str">
-        <f>VLOOKUP(A12,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B03.000.000</v>
+      <c r="A12" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>308</v>
-      </c>
-      <c r="B13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" t="s">
-        <v>107</v>
-      </c>
-      <c r="D13" t="str">
-        <f>VLOOKUP(A13,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B03.000.000</v>
+      <c r="A13" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>252</v>
-      </c>
-      <c r="B14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D14" t="str">
-        <f>VLOOKUP(A14,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B04.000.000</v>
+      <c r="A14" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>275</v>
-      </c>
-      <c r="B15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" t="s">
-        <v>141</v>
-      </c>
-      <c r="D15" t="str">
-        <f>VLOOKUP(A15,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B04.000.000</v>
+      <c r="A15" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" t="str">
-        <f>VLOOKUP(A16,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B05.000.000</v>
+      <c r="A16" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>287</v>
-      </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" t="str">
-        <f>VLOOKUP(A17,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B05.000.000</v>
+      <c r="A17" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>295</v>
-      </c>
-      <c r="B18" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" t="str">
-        <f>VLOOKUP(A18,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B05.000.000</v>
+      <c r="A18" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>261</v>
-      </c>
-      <c r="B19" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" t="s">
-        <v>111</v>
-      </c>
-      <c r="D19" t="str">
-        <f>VLOOKUP(A19,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B05.000.000</v>
+      <c r="A19" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>273</v>
-      </c>
-      <c r="B20" t="s">
-        <v>136</v>
-      </c>
-      <c r="C20" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" t="str">
-        <f>VLOOKUP(A20,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B05.000.000</v>
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>254</v>
-      </c>
-      <c r="B21" t="s">
-        <v>93</v>
-      </c>
-      <c r="C21" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" t="str">
-        <f>VLOOKUP(A21,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B07.000.000</v>
+      <c r="A21" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>256</v>
-      </c>
-      <c r="B22" t="s">
-        <v>97</v>
-      </c>
-      <c r="C22" t="s">
-        <v>98</v>
-      </c>
-      <c r="D22" t="str">
-        <f>VLOOKUP(A22,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B07.000.000</v>
+      <c r="A22" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>263</v>
-      </c>
-      <c r="B23" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" t="s">
-        <v>115</v>
-      </c>
-      <c r="D23" t="str">
-        <f>VLOOKUP(A23,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B08.000.000</v>
+      <c r="A23" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" t="str">
-        <f>VLOOKUP(A24,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B10.000.000</v>
+      <c r="A24" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>285</v>
-      </c>
-      <c r="B25" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" t="s">
-        <v>32</v>
-      </c>
-      <c r="D25" t="str">
-        <f>VLOOKUP(A25,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B10.000.000</v>
+      <c r="A25" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>270</v>
-      </c>
-      <c r="B26" t="s">
-        <v>130</v>
-      </c>
-      <c r="C26" t="s">
-        <v>131</v>
-      </c>
-      <c r="D26" t="str">
-        <f>VLOOKUP(A26,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B10.000.000</v>
+      <c r="A26" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>258</v>
-      </c>
-      <c r="B27" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" t="s">
-        <v>102</v>
-      </c>
-      <c r="D27" t="str">
-        <f>VLOOKUP(A27,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B12.000.000</v>
+      <c r="A27" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>259</v>
-      </c>
-      <c r="B28" t="s">
-        <v>104</v>
-      </c>
-      <c r="C28" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" t="str">
-        <f>VLOOKUP(A28,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B12.000.000</v>
+      <c r="A28" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>309</v>
-      </c>
-      <c r="B29" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" t="s">
-        <v>119</v>
-      </c>
-      <c r="D29" t="str">
-        <f>VLOOKUP(A29,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>B12.000.000</v>
+      <c r="A29" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>12</v>
-      </c>
-      <c r="B30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C30" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" t="str">
-        <f>VLOOKUP(A30,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C02.000.000</v>
+      <c r="A30" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>286</v>
-      </c>
-      <c r="B31" t="s">
-        <v>33</v>
-      </c>
-      <c r="C31" t="s">
-        <v>34</v>
-      </c>
-      <c r="D31" t="str">
-        <f>VLOOKUP(A31,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C04.000.000</v>
+      <c r="A31" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>262</v>
-      </c>
-      <c r="B32" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" t="s">
-        <v>113</v>
-      </c>
-      <c r="D32" t="str">
-        <f>VLOOKUP(A32,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C06.000.000</v>
+      <c r="A32" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>157</v>
-      </c>
-      <c r="B33" t="s">
-        <v>22</v>
-      </c>
-      <c r="C33" t="s">
-        <v>23</v>
-      </c>
-      <c r="D33" t="str">
-        <f>VLOOKUP(A33,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C08.000.000</v>
+      <c r="A33" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C34" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" t="str">
-        <f>VLOOKUP(A34,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C08.000.000</v>
+      <c r="A34" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>265</v>
-      </c>
-      <c r="B35" t="s">
-        <v>120</v>
-      </c>
-      <c r="C35" t="s">
-        <v>121</v>
-      </c>
-      <c r="D35" t="str">
-        <f>VLOOKUP(A35,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C08.000.000</v>
+      <c r="A35" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>289</v>
-      </c>
-      <c r="B36" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" t="str">
-        <f>VLOOKUP(A36,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A36" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>290</v>
-      </c>
-      <c r="B37" t="s">
-        <v>41</v>
-      </c>
-      <c r="C37" t="s">
-        <v>42</v>
-      </c>
-      <c r="D37" t="str">
-        <f>VLOOKUP(A37,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A37" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>291</v>
-      </c>
-      <c r="B38" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" t="s">
-        <v>45</v>
-      </c>
-      <c r="D38" t="str">
-        <f>VLOOKUP(A38,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A38" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>215</v>
-      </c>
-      <c r="B39" t="s">
-        <v>46</v>
-      </c>
-      <c r="C39" t="s">
-        <v>47</v>
-      </c>
-      <c r="D39" t="str">
-        <f>VLOOKUP(A39,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A39" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>292</v>
-      </c>
-      <c r="B40" t="s">
-        <v>48</v>
-      </c>
-      <c r="C40" t="s">
-        <v>49</v>
-      </c>
-      <c r="D40" t="str">
-        <f>VLOOKUP(A40,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A40" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>293</v>
-      </c>
-      <c r="B41" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" t="s">
-        <v>51</v>
-      </c>
-      <c r="D41" t="str">
-        <f>VLOOKUP(A41,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A41" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>218</v>
-      </c>
-      <c r="B42" t="s">
-        <v>52</v>
-      </c>
-      <c r="C42" t="s">
-        <v>53</v>
-      </c>
-      <c r="D42" t="str">
-        <f>VLOOKUP(A42,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A42" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>294</v>
-      </c>
-      <c r="B43" t="s">
-        <v>54</v>
-      </c>
-      <c r="C43" t="s">
-        <v>55</v>
-      </c>
-      <c r="D43" t="str">
-        <f>VLOOKUP(A43,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A43" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>219</v>
-      </c>
-      <c r="B44" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" t="str">
-        <f>VLOOKUP(A44,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A44" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>142</v>
-      </c>
-      <c r="B45" t="s">
-        <v>58</v>
-      </c>
-      <c r="C45" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" t="str">
-        <f>VLOOKUP(A45,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A45" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>296</v>
-      </c>
-      <c r="B46" t="s">
-        <v>62</v>
-      </c>
-      <c r="C46" t="s">
-        <v>63</v>
-      </c>
-      <c r="D46" t="str">
-        <f>VLOOKUP(A46,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A46" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>297</v>
-      </c>
-      <c r="B47" t="s">
-        <v>64</v>
-      </c>
-      <c r="C47" t="s">
-        <v>65</v>
-      </c>
-      <c r="D47" t="str">
-        <f>VLOOKUP(A47,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
+      <c r="A47" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>298</v>
-      </c>
-      <c r="B48" t="s">
-        <v>66</v>
-      </c>
-      <c r="C48" t="s">
-        <v>67</v>
-      </c>
-      <c r="D48" t="str">
-        <f>VLOOKUP(A48,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>251</v>
-      </c>
-      <c r="B49" t="s">
-        <v>68</v>
-      </c>
-      <c r="C49" t="s">
-        <v>69</v>
-      </c>
-      <c r="D49" t="str">
-        <f>VLOOKUP(A49,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>299</v>
-      </c>
-      <c r="B50" t="s">
-        <v>70</v>
-      </c>
-      <c r="C50" t="s">
-        <v>71</v>
-      </c>
-      <c r="D50" t="str">
-        <f>VLOOKUP(A50,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>301</v>
-      </c>
-      <c r="B51" t="s">
-        <v>74</v>
-      </c>
-      <c r="C51" t="s">
-        <v>75</v>
-      </c>
-      <c r="D51" t="str">
-        <f>VLOOKUP(A51,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>302</v>
-      </c>
-      <c r="B52" t="s">
-        <v>76</v>
-      </c>
-      <c r="C52" t="s">
-        <v>77</v>
-      </c>
-      <c r="D52" t="str">
-        <f>VLOOKUP(A52,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>303</v>
-      </c>
-      <c r="B53" t="s">
-        <v>78</v>
-      </c>
-      <c r="C53" t="s">
-        <v>79</v>
-      </c>
-      <c r="D53" t="str">
-        <f>VLOOKUP(A53,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>305</v>
-      </c>
-      <c r="B54" t="s">
-        <v>83</v>
-      </c>
-      <c r="C54" t="s">
-        <v>84</v>
-      </c>
-      <c r="D54" t="str">
-        <f>VLOOKUP(A54,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>306</v>
-      </c>
-      <c r="B55" t="s">
-        <v>85</v>
-      </c>
-      <c r="C55" t="s">
-        <v>86</v>
-      </c>
-      <c r="D55" t="str">
-        <f>VLOOKUP(A55,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>307</v>
-      </c>
-      <c r="B56" t="s">
-        <v>87</v>
-      </c>
-      <c r="C56" t="s">
-        <v>88</v>
-      </c>
-      <c r="D56" t="str">
-        <f>VLOOKUP(A56,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>C12.000.000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>282</v>
-      </c>
-      <c r="B57" t="s">
-        <v>8</v>
-      </c>
-      <c r="C57" t="s">
-        <v>9</v>
-      </c>
-      <c r="D57" t="str">
-        <f>VLOOKUP(A57,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>CAL.000.000</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>267</v>
-      </c>
-      <c r="B58" t="s">
-        <v>124</v>
-      </c>
-      <c r="C58" t="s">
-        <v>125</v>
-      </c>
-      <c r="D58" t="str">
-        <f>VLOOKUP(A58,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>CAL.000.000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>272</v>
-      </c>
-      <c r="B59" t="s">
-        <v>134</v>
-      </c>
-      <c r="C59" t="s">
-        <v>135</v>
-      </c>
-      <c r="D59" t="str">
-        <f>VLOOKUP(A59,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>CAL.000.000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>257</v>
-      </c>
-      <c r="B60" t="s">
-        <v>99</v>
-      </c>
-      <c r="C60" t="s">
-        <v>100</v>
-      </c>
-      <c r="D60" t="str">
-        <f>VLOOKUP(A60,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>CAL.TRA.NSP</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>281</v>
-      </c>
-      <c r="B61" t="s">
-        <v>6</v>
-      </c>
-      <c r="C61" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61" t="str">
-        <f>VLOOKUP(A61,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>PL4.000.000</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>276</v>
-      </c>
-      <c r="B62" t="s">
-        <v>144</v>
-      </c>
-      <c r="C62" t="s">
-        <v>145</v>
-      </c>
-      <c r="D62" t="str">
-        <f>VLOOKUP(A62,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>PL4.000.000</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>260</v>
-      </c>
-      <c r="B63" t="s">
-        <v>108</v>
-      </c>
-      <c r="C63" t="s">
-        <v>109</v>
-      </c>
-      <c r="D63" t="str">
-        <f>VLOOKUP(A63,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>SCR.OCA.SA</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>284</v>
-      </c>
-      <c r="B64" t="s">
-        <v>19</v>
-      </c>
-      <c r="C64" t="s">
-        <v>20</v>
-      </c>
-      <c r="D64" t="str">
-        <f>VLOOKUP(A64,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>SIN.000.000</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>288</v>
-      </c>
-      <c r="B65" t="s">
-        <v>37</v>
-      </c>
-      <c r="C65" t="s">
-        <v>38</v>
-      </c>
-      <c r="D65" t="str">
-        <f>VLOOKUP(A65,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>SIN.000.000</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>268</v>
-      </c>
-      <c r="B66" t="s">
-        <v>126</v>
-      </c>
-      <c r="C66" t="s">
-        <v>127</v>
-      </c>
-      <c r="D66" t="str">
-        <f>VLOOKUP(A66,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>SIN.000.000</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>271</v>
-      </c>
-      <c r="B67" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" t="s">
-        <v>133</v>
-      </c>
-      <c r="D67" t="str">
-        <f>VLOOKUP(A67,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
-        <v>SIN.000.000</v>
+      <c r="A48" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D67" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D67">
-      <sortCondition ref="D1:D67"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:D48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -25248,7 +24906,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>277</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -25256,10 +24914,10 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>152</v>
+        <v>88</v>
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP(A2,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25268,13 +24926,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>243</v>
+        <v>174</v>
       </c>
       <c r="B3" t="s">
-        <v>203</v>
+        <v>137</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>138</v>
       </c>
       <c r="D3" t="str">
         <f>VLOOKUP(A3,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25283,13 +24941,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>247</v>
+        <v>178</v>
       </c>
       <c r="B4" t="s">
-        <v>211</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>212</v>
+        <v>146</v>
       </c>
       <c r="D4" t="str">
         <f>VLOOKUP(A4,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25298,13 +24956,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>154</v>
+        <v>90</v>
       </c>
       <c r="D5" t="str">
         <f>VLOOKUP(A5,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25313,13 +24971,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>229</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="D6" t="str">
         <f>VLOOKUP(A6,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25328,13 +24986,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>239</v>
+        <v>170</v>
       </c>
       <c r="B7" t="s">
-        <v>195</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>196</v>
+        <v>130</v>
       </c>
       <c r="D7" t="str">
         <f>VLOOKUP(A7,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25343,13 +25001,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>241</v>
+        <v>172</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>133</v>
       </c>
       <c r="C8" t="s">
-        <v>200</v>
+        <v>134</v>
       </c>
       <c r="D8" t="str">
         <f>VLOOKUP(A8,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25358,13 +25016,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>250</v>
+        <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>222</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s">
-        <v>223</v>
+        <v>154</v>
       </c>
       <c r="D9" t="str">
         <f>VLOOKUP(A9,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25373,13 +25031,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>155</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
-        <v>156</v>
+        <v>92</v>
       </c>
       <c r="D10" t="str">
         <f>VLOOKUP(A10,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25388,13 +25046,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>227</v>
+        <v>158</v>
       </c>
       <c r="B11" t="s">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>106</v>
       </c>
       <c r="D11" t="str">
         <f>VLOOKUP(A11,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25403,13 +25061,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
-        <v>147</v>
+        <v>83</v>
       </c>
       <c r="C12" t="s">
-        <v>148</v>
+        <v>84</v>
       </c>
       <c r="D12" t="str">
         <f>VLOOKUP(A12,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25421,10 +25079,10 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>149</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
-        <v>150</v>
+        <v>86</v>
       </c>
       <c r="D13" t="str">
         <f>VLOOKUP(A13,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25433,13 +25091,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>233</v>
+        <v>164</v>
       </c>
       <c r="B14" t="s">
-        <v>183</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
-        <v>184</v>
+        <v>118</v>
       </c>
       <c r="D14" t="str">
         <f>VLOOKUP(A14,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25448,13 +25106,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>242</v>
+        <v>173</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>135</v>
       </c>
       <c r="C15" t="s">
-        <v>202</v>
+        <v>136</v>
       </c>
       <c r="D15" t="str">
         <f>VLOOKUP(A15,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25463,13 +25121,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>246</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>209</v>
+        <v>143</v>
       </c>
       <c r="C16" t="s">
-        <v>210</v>
+        <v>144</v>
       </c>
       <c r="D16" t="str">
         <f>VLOOKUP(A16,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25478,13 +25136,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>226</v>
+        <v>157</v>
       </c>
       <c r="B17" t="s">
-        <v>169</v>
+        <v>103</v>
       </c>
       <c r="C17" t="s">
-        <v>170</v>
+        <v>104</v>
       </c>
       <c r="D17" t="str">
         <f>VLOOKUP(A17,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25493,13 +25151,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>249</v>
+        <v>180</v>
       </c>
       <c r="B18" t="s">
-        <v>216</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>217</v>
+        <v>150</v>
       </c>
       <c r="D18" t="str">
         <f>VLOOKUP(A18,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25508,13 +25166,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>244</v>
+        <v>175</v>
       </c>
       <c r="B19" t="s">
-        <v>205</v>
+        <v>139</v>
       </c>
       <c r="C19" t="s">
-        <v>206</v>
+        <v>140</v>
       </c>
       <c r="D19" t="str">
         <f>VLOOKUP(A19,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25523,13 +25181,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>237</v>
+        <v>168</v>
       </c>
       <c r="B20" t="s">
-        <v>191</v>
+        <v>125</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>126</v>
       </c>
       <c r="D20" t="str">
         <f>VLOOKUP(A20,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25538,13 +25196,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>248</v>
+        <v>179</v>
       </c>
       <c r="B21" t="s">
-        <v>213</v>
+        <v>147</v>
       </c>
       <c r="C21" t="s">
-        <v>214</v>
+        <v>148</v>
       </c>
       <c r="D21" t="str">
         <f>VLOOKUP(A21,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25553,13 +25211,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>230</v>
+        <v>161</v>
       </c>
       <c r="B22" t="s">
-        <v>177</v>
+        <v>111</v>
       </c>
       <c r="C22" t="s">
-        <v>178</v>
+        <v>112</v>
       </c>
       <c r="D22" t="str">
         <f>VLOOKUP(A22,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25568,13 +25226,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="B23" t="s">
-        <v>179</v>
+        <v>113</v>
       </c>
       <c r="C23" t="s">
-        <v>180</v>
+        <v>114</v>
       </c>
       <c r="D23" t="str">
         <f>VLOOKUP(A23,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25583,13 +25241,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>280</v>
+        <v>198</v>
       </c>
       <c r="B24" t="s">
-        <v>220</v>
+        <v>151</v>
       </c>
       <c r="C24" t="s">
-        <v>221</v>
+        <v>152</v>
       </c>
       <c r="D24" t="str">
         <f>VLOOKUP(A24,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25598,13 +25256,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>278</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>158</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>159</v>
+        <v>94</v>
       </c>
       <c r="D25" t="str">
         <f>VLOOKUP(A25,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25613,13 +25271,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>143</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="C26" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="D26" t="str">
         <f>VLOOKUP(A26,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25628,13 +25286,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>224</v>
+        <v>155</v>
       </c>
       <c r="B27" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>98</v>
       </c>
       <c r="D27" t="str">
         <f>VLOOKUP(A27,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25643,13 +25301,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>279</v>
+        <v>197</v>
       </c>
       <c r="B28" t="s">
-        <v>165</v>
+        <v>99</v>
       </c>
       <c r="C28" t="s">
-        <v>166</v>
+        <v>100</v>
       </c>
       <c r="D28" t="str">
         <f>VLOOKUP(A28,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25658,13 +25316,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>240</v>
+        <v>171</v>
       </c>
       <c r="B29" t="s">
-        <v>197</v>
+        <v>131</v>
       </c>
       <c r="C29" t="s">
-        <v>198</v>
+        <v>132</v>
       </c>
       <c r="D29" t="str">
         <f>VLOOKUP(A29,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25673,13 +25331,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>245</v>
+        <v>176</v>
       </c>
       <c r="B30" t="s">
-        <v>207</v>
+        <v>141</v>
       </c>
       <c r="C30" t="s">
-        <v>208</v>
+        <v>142</v>
       </c>
       <c r="D30" t="str">
         <f>VLOOKUP(A30,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25688,13 +25346,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="B31" t="s">
-        <v>189</v>
+        <v>123</v>
       </c>
       <c r="C31" t="s">
-        <v>190</v>
+        <v>124</v>
       </c>
       <c r="D31" t="str">
         <f>VLOOKUP(A31,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25703,13 +25361,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>225</v>
+        <v>156</v>
       </c>
       <c r="B32" t="s">
-        <v>167</v>
+        <v>101</v>
       </c>
       <c r="C32" t="s">
-        <v>168</v>
+        <v>102</v>
       </c>
       <c r="D32" t="str">
         <f>VLOOKUP(A32,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25718,13 +25376,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>228</v>
+        <v>159</v>
       </c>
       <c r="B33" t="s">
-        <v>173</v>
+        <v>107</v>
       </c>
       <c r="C33" t="s">
-        <v>174</v>
+        <v>108</v>
       </c>
       <c r="D33" t="str">
         <f>VLOOKUP(A33,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25733,13 +25391,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>232</v>
+        <v>163</v>
       </c>
       <c r="B34" t="s">
-        <v>181</v>
+        <v>115</v>
       </c>
       <c r="C34" t="s">
-        <v>182</v>
+        <v>116</v>
       </c>
       <c r="D34" t="str">
         <f>VLOOKUP(A34,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25748,13 +25406,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>234</v>
+        <v>165</v>
       </c>
       <c r="B35" t="s">
-        <v>185</v>
+        <v>119</v>
       </c>
       <c r="C35" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="D35" t="str">
         <f>VLOOKUP(A35,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25763,13 +25421,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>235</v>
+        <v>166</v>
       </c>
       <c r="B36" t="s">
-        <v>187</v>
+        <v>121</v>
       </c>
       <c r="C36" t="s">
-        <v>188</v>
+        <v>122</v>
       </c>
       <c r="D36" t="str">
         <f>VLOOKUP(A36,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>
@@ -25778,13 +25436,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>238</v>
+        <v>169</v>
       </c>
       <c r="B37" t="s">
-        <v>193</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s">
-        <v>194</v>
+        <v>128</v>
       </c>
       <c r="D37" t="str">
         <f>VLOOKUP(A37,[1]XXINRSAR_143999612_1!$A$1:$I$789,9,FALSE)</f>

</xml_diff>